<commit_message>
fix Authorization file set
</commit_message>
<xml_diff>
--- a/docs/JMeter_Usage_Guide.xlsx
+++ b/docs/JMeter_Usage_Guide.xlsx
@@ -23,12 +23,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="1052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="1059">
   <si>
     <t>JMeter APIテスト 利用方法</t>
   </si>
   <si>
-    <t>対象: Apache JMeter 5.6.3 ／ RHEL 9.8 ／ Windows 11 ／ ツール: jmeter_api_tool v1.0.0（2026-10-11 出力）</t>
+    <t>対象: Apache JMeter 5.6.3 ／ RHEL 9.8 ／ Windows 11 ／ ツール: jmeter_api_tool v1.0.0（2026-10-24 出力）</t>
   </si>
   <si>
     <t>本書は、REST API の定義（URL・HTTPメソッド・クエリパラメータ・ヘッダ・リクエストボディ）を Excel または CSV に記入し、JMeter のテスト計画ファイル（JMX）を自動生成して実行し、結果を確認するまでの手順をまとめたものです。</t>
@@ -782,6 +782,27 @@
   </si>
   <si>
     <t>全 API に付けるヘッダ。「名前: 値」を改行区切り（テンプレートの記入例: Accept: application/json / User-Agent: JMeter-API-Test/1.0 / X-Client-Id: ${CLIENT_ID}）</t>
+  </si>
+  <si>
+    <t>access_token_dir</t>
+  </si>
+  <si>
+    <t>アクセストークンのフォルダ</t>
+  </si>
+  <si>
+    <t>指定すると、このフォルダ配下のファイルからアクセストークンを読み込み、共通ヘッダに Authorization: Bearer ${ACCESS_TOKEN} を付けます（共通ヘッダに Authorization がある場合はその値を使用）。空欄 = 使わない。JMX からの相対パスまたは絶対パス。-JACCESS_TOKEN_DIR</t>
+  </si>
+  <si>
+    <t>access_token_file</t>
+  </si>
+  <si>
+    <t>アクセストークンのファイル名</t>
+  </si>
+  <si>
+    <t>access_token.txt</t>
+  </si>
+  <si>
+    <t>アクセストークンを書いたファイルの名前（フォルダからの相対パス）。前後の空白・改行は除き、実行中にファイルが更新されると読み直します。-JACCESS_TOKEN_FILE</t>
   </si>
   <si>
     <t>follow_redirects</t>
@@ -3800,50 +3821,50 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>794</v>
+        <v>801</v>
       </c>
       <c r="C3" s="4"/>
     </row>
     <row r="4" ht="4" customHeight="1"/>
     <row r="5" ht="16.2" customHeight="1">
       <c r="B5" s="9" t="s">
-        <v>795</v>
+        <v>802</v>
       </c>
       <c r="C5" s="9"/>
     </row>
     <row r="6" ht="16.2" customHeight="1">
       <c r="B6" s="10" t="s">
-        <v>796</v>
+        <v>803</v>
       </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" ht="16.2" customHeight="1">
       <c r="B7" s="10" t="s">
-        <v>797</v>
+        <v>804</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" ht="16.2" customHeight="1">
       <c r="B8" s="10" t="s">
-        <v>798</v>
+        <v>805</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" ht="16.2" customHeight="1">
       <c r="B9" s="10" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" ht="16.2" customHeight="1">
       <c r="B10" s="10" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" ht="16.2" customHeight="1">
       <c r="B11" s="11" t="s">
-        <v>801</v>
+        <v>808</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -3851,55 +3872,55 @@
     <row r="13" ht="8" customHeight="1"/>
     <row r="14" ht="24" customHeight="1">
       <c r="B14" s="4" t="s">
-        <v>802</v>
+        <v>809</v>
       </c>
       <c r="C14" s="4"/>
     </row>
     <row r="15" ht="4" customHeight="1"/>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="13" t="s">
-        <v>803</v>
+        <v>810</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>804</v>
+        <v>811</v>
       </c>
     </row>
     <row r="17" ht="32.4" customHeight="1">
       <c r="B17" s="14" t="s">
-        <v>805</v>
+        <v>812</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>806</v>
+        <v>813</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="15" t="s">
-        <v>807</v>
+        <v>814</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>808</v>
+        <v>815</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="14" t="s">
-        <v>809</v>
+        <v>816</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>810</v>
+        <v>817</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="s">
-        <v>811</v>
+        <v>818</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>812</v>
+        <v>819</v>
       </c>
     </row>
     <row r="21" ht="6" customHeight="1"/>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="6" t="s">
-        <v>813</v>
+        <v>820</v>
       </c>
       <c r="C22" s="6"/>
     </row>
@@ -3907,14 +3928,14 @@
     <row r="24" ht="8" customHeight="1"/>
     <row r="25" ht="24" customHeight="1">
       <c r="B25" s="4" t="s">
-        <v>814</v>
+        <v>821</v>
       </c>
       <c r="C25" s="4"/>
     </row>
     <row r="26" ht="4" customHeight="1"/>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="13" t="s">
-        <v>815</v>
+        <v>822</v>
       </c>
       <c r="C27" s="13" t="s">
         <v>6</v>
@@ -3922,104 +3943,104 @@
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="14" t="s">
-        <v>816</v>
+        <v>823</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>817</v>
+        <v>824</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="15" t="s">
-        <v>818</v>
+        <v>825</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>819</v>
+        <v>826</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="14" t="s">
-        <v>820</v>
+        <v>827</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>821</v>
+        <v>828</v>
       </c>
     </row>
     <row r="31" ht="32.4" customHeight="1">
       <c r="B31" s="15" t="s">
-        <v>822</v>
+        <v>829</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>823</v>
+        <v>830</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="14" t="s">
-        <v>824</v>
+        <v>831</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>825</v>
+        <v>832</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="15" t="s">
-        <v>826</v>
+        <v>833</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>827</v>
+        <v>834</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="14" t="s">
-        <v>828</v>
+        <v>835</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>829</v>
+        <v>836</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="15" t="s">
-        <v>830</v>
+        <v>837</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>831</v>
+        <v>838</v>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="14" t="s">
-        <v>832</v>
+        <v>839</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>833</v>
+        <v>840</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="15" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>834</v>
+        <v>841</v>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="14" t="s">
-        <v>835</v>
+        <v>842</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>836</v>
+        <v>843</v>
       </c>
     </row>
     <row r="39" ht="6" customHeight="1"/>
     <row r="40" ht="8" customHeight="1"/>
     <row r="41" ht="24" customHeight="1">
       <c r="B41" s="4" t="s">
-        <v>837</v>
+        <v>844</v>
       </c>
       <c r="C41" s="4"/>
     </row>
     <row r="42" ht="4" customHeight="1"/>
     <row r="43" ht="46.8" customHeight="1">
       <c r="B43" s="6" t="s">
-        <v>838</v>
+        <v>845</v>
       </c>
       <c r="C43" s="6"/>
     </row>
@@ -4027,14 +4048,14 @@
     <row r="45" ht="8" customHeight="1"/>
     <row r="46" ht="24" customHeight="1">
       <c r="B46" s="4" t="s">
-        <v>839</v>
+        <v>846</v>
       </c>
       <c r="C46" s="4"/>
     </row>
     <row r="47" ht="4" customHeight="1"/>
     <row r="48" ht="32.4" customHeight="1">
       <c r="B48" s="6" t="s">
-        <v>840</v>
+        <v>847</v>
       </c>
       <c r="C48" s="6"/>
     </row>
@@ -4042,26 +4063,26 @@
     <row r="50" ht="8" customHeight="1"/>
     <row r="51" ht="24" customHeight="1">
       <c r="B51" s="4" t="s">
-        <v>841</v>
+        <v>848</v>
       </c>
       <c r="C51" s="4"/>
     </row>
     <row r="52" ht="4" customHeight="1"/>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="7" t="s">
-        <v>842</v>
+        <v>849</v>
       </c>
       <c r="C53" s="7"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="7" t="s">
-        <v>843</v>
+        <v>850</v>
       </c>
       <c r="C54" s="7"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="7" t="s">
-        <v>844</v>
+        <v>851</v>
       </c>
       <c r="C55" s="7"/>
     </row>
@@ -4121,7 +4142,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>845</v>
+        <v>852</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -4129,10 +4150,10 @@
     <row r="4" ht="4" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>6</v>
@@ -4140,97 +4161,97 @@
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="14" t="s">
-        <v>846</v>
+        <v>853</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>847</v>
+        <v>854</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>848</v>
+        <v>855</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>849</v>
+        <v>856</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>850</v>
+        <v>857</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>851</v>
+        <v>858</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="15" t="s">
-        <v>852</v>
+        <v>859</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>853</v>
+        <v>860</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>854</v>
+        <v>861</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>855</v>
+        <v>862</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="15" t="s">
-        <v>856</v>
+        <v>863</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>857</v>
+        <v>864</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>858</v>
+        <v>865</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>859</v>
+        <v>866</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>860</v>
+        <v>867</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="15" t="s">
-        <v>861</v>
+        <v>868</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>862</v>
+        <v>869</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>863</v>
+        <v>870</v>
       </c>
     </row>
     <row r="14" ht="6" customHeight="1"/>
     <row r="15" ht="8" customHeight="1"/>
     <row r="16" ht="24" customHeight="1">
       <c r="B16" s="4" t="s">
-        <v>864</v>
+        <v>871</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
@@ -4238,152 +4259,152 @@
     <row r="17" ht="4" customHeight="1"/>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="13" t="s">
-        <v>865</v>
+        <v>872</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>866</v>
+        <v>873</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="14" t="s">
-        <v>867</v>
+        <v>874</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>868</v>
+        <v>875</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>869</v>
+        <v>876</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="15" t="s">
-        <v>870</v>
+        <v>877</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>871</v>
+        <v>878</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>872</v>
+        <v>879</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="14" t="s">
-        <v>873</v>
+        <v>880</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>874</v>
+        <v>881</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>875</v>
+        <v>882</v>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="15" t="s">
-        <v>876</v>
+        <v>883</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>877</v>
+        <v>884</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>878</v>
+        <v>885</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="14" t="s">
-        <v>879</v>
+        <v>886</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>880</v>
+        <v>887</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>881</v>
+        <v>888</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="15" t="s">
-        <v>882</v>
+        <v>889</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>883</v>
+        <v>890</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>884</v>
+        <v>891</v>
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="14" t="s">
-        <v>885</v>
+        <v>892</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>886</v>
+        <v>893</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>887</v>
+        <v>894</v>
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="15" t="s">
-        <v>888</v>
+        <v>895</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>889</v>
+        <v>896</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>890</v>
+        <v>897</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="14" t="s">
-        <v>891</v>
+        <v>898</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>892</v>
+        <v>899</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>893</v>
+        <v>900</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="s">
-        <v>894</v>
+        <v>901</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>895</v>
+        <v>902</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>896</v>
+        <v>903</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="14" t="s">
-        <v>897</v>
+        <v>904</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>898</v>
+        <v>905</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>899</v>
+        <v>906</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="s">
-        <v>900</v>
+        <v>907</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>901</v>
+        <v>908</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>902</v>
+        <v>909</v>
       </c>
     </row>
     <row r="31" ht="6" customHeight="1"/>
     <row r="32" ht="8" customHeight="1"/>
     <row r="33" ht="24" customHeight="1">
       <c r="B33" s="4" t="s">
-        <v>903</v>
+        <v>910</v>
       </c>
       <c r="C33" s="4"/>
       <c r="D33" s="4"/>
@@ -4391,21 +4412,21 @@
     <row r="34" ht="4" customHeight="1"/>
     <row r="35" ht="16.2" customHeight="1">
       <c r="B35" s="9" t="s">
-        <v>904</v>
+        <v>911</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
     </row>
     <row r="36" ht="16.2" customHeight="1">
       <c r="B36" s="10" t="s">
-        <v>905</v>
+        <v>912</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
     </row>
     <row r="37" ht="16.2" customHeight="1">
       <c r="B37" s="10" t="s">
-        <v>906</v>
+        <v>913</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
@@ -4419,21 +4440,21 @@
     </row>
     <row r="39" ht="16.2" customHeight="1">
       <c r="B39" s="10" t="s">
-        <v>907</v>
+        <v>914</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" ht="16.2" customHeight="1">
       <c r="B40" s="10" t="s">
-        <v>908</v>
+        <v>915</v>
       </c>
       <c r="C40" s="10"/>
       <c r="D40" s="10"/>
     </row>
     <row r="41" ht="16.2" customHeight="1">
       <c r="B41" s="10" t="s">
-        <v>909</v>
+        <v>916</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="10"/>
@@ -4447,28 +4468,28 @@
     </row>
     <row r="43" ht="16.2" customHeight="1">
       <c r="B43" s="10" t="s">
-        <v>910</v>
+        <v>917</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="10"/>
     </row>
     <row r="44" ht="16.2" customHeight="1">
       <c r="B44" s="10" t="s">
-        <v>911</v>
+        <v>918</v>
       </c>
       <c r="C44" s="10"/>
       <c r="D44" s="10"/>
     </row>
     <row r="45" ht="16.2" customHeight="1">
       <c r="B45" s="10" t="s">
-        <v>912</v>
+        <v>919</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="10"/>
     </row>
     <row r="46" ht="16.2" customHeight="1">
       <c r="B46" s="10" t="s">
-        <v>913</v>
+        <v>920</v>
       </c>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
@@ -4482,14 +4503,14 @@
     </row>
     <row r="48" ht="16.2" customHeight="1">
       <c r="B48" s="10" t="s">
-        <v>914</v>
+        <v>921</v>
       </c>
       <c r="C48" s="10"/>
       <c r="D48" s="10"/>
     </row>
     <row r="49" ht="16.2" customHeight="1">
       <c r="B49" s="11" t="s">
-        <v>915</v>
+        <v>922</v>
       </c>
       <c r="C49" s="11"/>
       <c r="D49" s="11"/>
@@ -4497,21 +4518,21 @@
     <row r="50" ht="6" customHeight="1"/>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="7" t="s">
-        <v>916</v>
+        <v>923</v>
       </c>
       <c r="C51" s="7"/>
       <c r="D51" s="7"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="7" t="s">
-        <v>917</v>
+        <v>924</v>
       </c>
       <c r="C52" s="7"/>
       <c r="D52" s="7"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="7" t="s">
-        <v>918</v>
+        <v>925</v>
       </c>
       <c r="C53" s="7"/>
       <c r="D53" s="7"/>
@@ -4520,7 +4541,7 @@
     <row r="55" ht="8" customHeight="1"/>
     <row r="56" ht="24" customHeight="1">
       <c r="B56" s="4" t="s">
-        <v>919</v>
+        <v>926</v>
       </c>
       <c r="C56" s="4"/>
       <c r="D56" s="4"/>
@@ -4528,60 +4549,60 @@
     <row r="57" ht="4" customHeight="1"/>
     <row r="58" ht="18" customHeight="1">
       <c r="B58" s="13" t="s">
-        <v>920</v>
+        <v>927</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>921</v>
+        <v>928</v>
       </c>
       <c r="D58" s="13"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="B59" s="14" t="s">
-        <v>922</v>
+        <v>929</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>923</v>
+        <v>930</v>
       </c>
       <c r="D59" s="14"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="B60" s="15" t="s">
-        <v>924</v>
+        <v>931</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>925</v>
+        <v>932</v>
       </c>
       <c r="D60" s="15"/>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="B61" s="14" t="s">
-        <v>926</v>
+        <v>933</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>927</v>
+        <v>934</v>
       </c>
       <c r="D61" s="14"/>
     </row>
     <row r="62" ht="32.4" customHeight="1">
       <c r="B62" s="15" t="s">
-        <v>928</v>
+        <v>935</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>929</v>
+        <v>936</v>
       </c>
       <c r="D62" s="15"/>
     </row>
     <row r="63" ht="6" customHeight="1"/>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="7" t="s">
-        <v>930</v>
+        <v>937</v>
       </c>
       <c r="C64" s="7"/>
       <c r="D64" s="7"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="7" t="s">
-        <v>931</v>
+        <v>938</v>
       </c>
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
@@ -4590,7 +4611,7 @@
     <row r="67" ht="8" customHeight="1"/>
     <row r="68" ht="24" customHeight="1">
       <c r="B68" s="4" t="s">
-        <v>932</v>
+        <v>939</v>
       </c>
       <c r="C68" s="4"/>
       <c r="D68" s="4"/>
@@ -4598,55 +4619,55 @@
     <row r="69" ht="4" customHeight="1"/>
     <row r="70" ht="18" customHeight="1">
       <c r="B70" s="13" t="s">
-        <v>920</v>
+        <v>927</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>933</v>
+        <v>940</v>
       </c>
       <c r="D70" s="13"/>
     </row>
     <row r="71" ht="18" customHeight="1">
       <c r="B71" s="14" t="s">
-        <v>934</v>
+        <v>941</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>935</v>
+        <v>942</v>
       </c>
       <c r="D71" s="14"/>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="B72" s="15" t="s">
-        <v>936</v>
+        <v>943</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>937</v>
+        <v>944</v>
       </c>
       <c r="D72" s="15"/>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="B73" s="14" t="s">
-        <v>938</v>
+        <v>945</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>939</v>
+        <v>946</v>
       </c>
       <c r="D73" s="14"/>
     </row>
     <row r="74" ht="18" customHeight="1">
       <c r="B74" s="15" t="s">
-        <v>940</v>
+        <v>947</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>941</v>
+        <v>948</v>
       </c>
       <c r="D74" s="15"/>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="B75" s="14" t="s">
-        <v>942</v>
+        <v>949</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>943</v>
+        <v>950</v>
       </c>
       <c r="D75" s="14"/>
     </row>
@@ -4723,200 +4744,200 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="13" t="s">
-        <v>944</v>
+        <v>951</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>945</v>
+        <v>952</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>946</v>
+        <v>953</v>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="14" t="s">
-        <v>947</v>
+        <v>954</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>948</v>
+        <v>955</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>949</v>
+        <v>956</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="15" t="s">
-        <v>950</v>
+        <v>957</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>951</v>
+        <v>958</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>952</v>
+        <v>959</v>
       </c>
     </row>
     <row r="6" ht="32.4" customHeight="1">
       <c r="B6" s="14" t="s">
-        <v>953</v>
+        <v>960</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>954</v>
+        <v>961</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>955</v>
+        <v>962</v>
       </c>
     </row>
     <row r="7" ht="32.4" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>956</v>
+        <v>963</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>957</v>
+        <v>964</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>958</v>
+        <v>965</v>
       </c>
     </row>
     <row r="8" ht="32.4" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>959</v>
+        <v>966</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>960</v>
+        <v>967</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>961</v>
+        <v>968</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="15" t="s">
-        <v>962</v>
+        <v>969</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>963</v>
+        <v>970</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>964</v>
+        <v>971</v>
       </c>
     </row>
     <row r="10" ht="32.4" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>965</v>
+        <v>972</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>966</v>
+        <v>973</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>967</v>
+        <v>974</v>
       </c>
     </row>
     <row r="11" ht="32.4" customHeight="1">
       <c r="B11" s="15" t="s">
-        <v>968</v>
+        <v>975</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>969</v>
+        <v>976</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>970</v>
+        <v>977</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>971</v>
+        <v>978</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>972</v>
+        <v>979</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>973</v>
+        <v>980</v>
       </c>
     </row>
     <row r="13" ht="32.4" customHeight="1">
       <c r="B13" s="15" t="s">
-        <v>974</v>
+        <v>981</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>975</v>
+        <v>982</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>976</v>
+        <v>983</v>
       </c>
     </row>
     <row r="14" ht="32.4" customHeight="1">
       <c r="B14" s="14" t="s">
-        <v>977</v>
+        <v>984</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>978</v>
+        <v>985</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>979</v>
+        <v>986</v>
       </c>
     </row>
     <row r="15" ht="32.4" customHeight="1">
       <c r="B15" s="15" t="s">
-        <v>980</v>
+        <v>987</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>981</v>
+        <v>988</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>982</v>
+        <v>989</v>
       </c>
     </row>
     <row r="16" ht="32.4" customHeight="1">
       <c r="B16" s="14" t="s">
-        <v>983</v>
+        <v>990</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>984</v>
+        <v>991</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>985</v>
+        <v>992</v>
       </c>
     </row>
     <row r="17" ht="32.4" customHeight="1">
       <c r="B17" s="15" t="s">
-        <v>986</v>
+        <v>993</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>987</v>
+        <v>994</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>988</v>
+        <v>995</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="14" t="s">
-        <v>989</v>
+        <v>996</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>990</v>
+        <v>997</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>991</v>
+        <v>998</v>
       </c>
     </row>
     <row r="19" ht="32.4" customHeight="1">
       <c r="B19" s="15" t="s">
-        <v>992</v>
+        <v>999</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>993</v>
+        <v>1000</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>994</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="20" ht="32.4" customHeight="1">
       <c r="B20" s="14" t="s">
-        <v>995</v>
+        <v>1002</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>996</v>
+        <v>1003</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>997</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="21" ht="6" customHeight="1"/>
@@ -4958,7 +4979,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>998</v>
+        <v>1005</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -4967,13 +4988,13 @@
     <row r="4" ht="4" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>999</v>
+        <v>1006</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>1000</v>
+        <v>1007</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>1001</v>
+        <v>1008</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>161</v>
@@ -4981,79 +5002,79 @@
     </row>
     <row r="6" ht="32.4" customHeight="1">
       <c r="B6" s="14" t="s">
-        <v>1002</v>
+        <v>1009</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1003</v>
+        <v>1010</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1004</v>
+        <v>1011</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1005</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="7" ht="32.4" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>1006</v>
+        <v>1013</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>1007</v>
+        <v>1014</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>1008</v>
+        <v>1015</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>1009</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="8" ht="32.4" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>1010</v>
+        <v>1017</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1011</v>
+        <v>1018</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1012</v>
+        <v>1019</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1013</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="15" t="s">
-        <v>1014</v>
+        <v>1021</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>1015</v>
+        <v>1022</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>1016</v>
+        <v>1023</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>1017</v>
+        <v>1024</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>1018</v>
+        <v>1025</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>134</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>1019</v>
+        <v>1026</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1020</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="11" ht="6" customHeight="1"/>
     <row r="12" ht="8" customHeight="1"/>
     <row r="13" ht="24" customHeight="1">
       <c r="B13" s="4" t="s">
-        <v>1021</v>
+        <v>1028</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
@@ -5062,7 +5083,7 @@
     <row r="14" ht="4" customHeight="1"/>
     <row r="15" ht="18" customHeight="1">
       <c r="B15" s="13" t="s">
-        <v>1022</v>
+        <v>1029</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>161</v>
@@ -5072,50 +5093,50 @@
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="B16" s="14" t="s">
-        <v>1023</v>
+        <v>1030</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>1024</v>
+        <v>1031</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="15" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>1025</v>
+        <v>1032</v>
       </c>
       <c r="D17" s="15"/>
       <c r="E17" s="15"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="14" t="s">
-        <v>1026</v>
+        <v>1033</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>1027</v>
+        <v>1034</v>
       </c>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="15" t="s">
-        <v>1028</v>
+        <v>1035</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>1029</v>
+        <v>1036</v>
       </c>
       <c r="D19" s="15"/>
       <c r="E19" s="15"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="14" t="s">
-        <v>1030</v>
+        <v>1037</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>1031</v>
+        <v>1038</v>
       </c>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
@@ -5125,7 +5146,7 @@
         <v>168</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>1032</v>
+        <v>1039</v>
       </c>
       <c r="D21" s="15"/>
       <c r="E21" s="15"/>
@@ -5135,97 +5156,97 @@
         <v>174</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>1033</v>
+        <v>1040</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="15" t="s">
-        <v>1034</v>
+        <v>1041</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>1035</v>
+        <v>1042</v>
       </c>
       <c r="D23" s="15"/>
       <c r="E23" s="15"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="B24" s="14" t="s">
-        <v>1036</v>
+        <v>1043</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>1037</v>
+        <v>1044</v>
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="B25" s="15" t="s">
-        <v>1038</v>
+        <v>1045</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>1039</v>
+        <v>1046</v>
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="B26" s="14" t="s">
-        <v>1040</v>
+        <v>1047</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>1041</v>
+        <v>1048</v>
       </c>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="15" t="s">
-        <v>1042</v>
+        <v>1049</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>1043</v>
+        <v>1050</v>
       </c>
       <c r="D27" s="15"/>
       <c r="E27" s="15"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="14" t="s">
-        <v>1044</v>
+        <v>1051</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>1045</v>
+        <v>1052</v>
       </c>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="15" t="s">
-        <v>1046</v>
+        <v>1053</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>1047</v>
+        <v>1054</v>
       </c>
       <c r="D29" s="15"/>
       <c r="E29" s="15"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="14" t="s">
-        <v>1048</v>
+        <v>1055</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>1049</v>
+        <v>1056</v>
       </c>
       <c r="D30" s="14"/>
       <c r="E30" s="14"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="15" t="s">
-        <v>1050</v>
+        <v>1057</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>1051</v>
+        <v>1058</v>
       </c>
       <c r="D31" s="15"/>
       <c r="E31" s="15"/>
@@ -6368,7 +6389,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -6690,7 +6711,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
+    <row r="24" ht="61.2" customHeight="1">
       <c r="B24" s="15" t="s">
         <v>237</v>
       </c>
@@ -6701,24 +6722,24 @@
         <v>254</v>
       </c>
       <c r="E24" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="F24" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
+    </row>
+    <row r="25" ht="46.8" customHeight="1">
       <c r="B25" s="14" t="s">
         <v>237</v>
       </c>
       <c r="C25" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="D25" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="E25" s="14" t="s">
         <v>258</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>255</v>
       </c>
       <c r="F25" s="14" t="s">
         <v>259</v>
@@ -6743,75 +6764,75 @@
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="B27" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="D27" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="E27" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="F27" s="14" t="s">
         <v>266</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="15" t="s">
-        <v>264</v>
+        <v>237</v>
       </c>
       <c r="C28" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>268</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="E28" s="15" t="s">
         <v>269</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>255</v>
       </c>
       <c r="F28" s="15" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="29" ht="32.4" customHeight="1">
+    <row r="29" ht="18" customHeight="1">
       <c r="B29" s="14" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>206</v>
+        <v>262</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" ht="32.4" customHeight="1">
       <c r="B31" s="14" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C31" s="14" t="s">
         <v>278</v>
@@ -6828,7 +6849,7 @@
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="15" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>281</v>
@@ -6837,24 +6858,24 @@
         <v>282</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>240</v>
+        <v>206</v>
       </c>
       <c r="F32" s="15" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
+    <row r="33" ht="32.4" customHeight="1">
       <c r="B33" s="14" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>286</v>
+        <v>206</v>
       </c>
       <c r="F33" s="14" t="s">
         <v>287</v>
@@ -6862,7 +6883,7 @@
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="15" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>288</v>
@@ -6871,71 +6892,71 @@
         <v>289</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F34" s="15"/>
+        <v>240</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>290</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="14" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="F35" s="14"/>
+        <v>293</v>
+      </c>
+      <c r="F35" s="14" t="s">
+        <v>294</v>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="B36" s="15" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>294</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>295</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F36" s="15"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="14" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>299</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F37" s="14"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="B38" s="15" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C38" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="D38" s="15" t="s">
         <v>300</v>
       </c>
-      <c r="D38" s="15" t="s">
+      <c r="E38" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="E38" s="15" t="s">
-        <v>240</v>
       </c>
       <c r="F38" s="15" t="s">
         <v>302</v>
@@ -6943,7 +6964,7 @@
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="14" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C39" s="14" t="s">
         <v>303</v>
@@ -6954,58 +6975,60 @@
       <c r="E39" s="14" t="s">
         <v>305</v>
       </c>
-      <c r="F39" s="14"/>
+      <c r="F39" s="14" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="15" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F40" s="15"/>
+        <v>240</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="14" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F41" s="14"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="B42" s="15" t="s">
-        <v>311</v>
+        <v>284</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>240</v>
-      </c>
-      <c r="F42" s="15" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="43" ht="32.4" customHeight="1">
+        <v>7</v>
+      </c>
+      <c r="F42" s="15"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
       <c r="B43" s="14" t="s">
-        <v>311</v>
+        <v>284</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>315</v>
@@ -7016,13 +7039,11 @@
       <c r="E43" s="14" t="s">
         <v>317</v>
       </c>
-      <c r="F43" s="14" t="s">
-        <v>318</v>
-      </c>
+      <c r="F43" s="14"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="15" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>319</v>
@@ -7031,15 +7052,15 @@
         <v>320</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="F44" s="15" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="45" ht="18" customHeight="1">
+    <row r="45" ht="32.4" customHeight="1">
       <c r="B45" s="14" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>322</v>
@@ -7048,71 +7069,71 @@
         <v>323</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="F45" s="14"/>
+        <v>324</v>
+      </c>
+      <c r="F45" s="14" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="15" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>326</v>
-      </c>
-      <c r="F46" s="15"/>
+        <v>206</v>
+      </c>
+      <c r="F46" s="15" t="s">
+        <v>328</v>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="14" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>329</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="F47" s="14"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="15" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>298</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="49" ht="32.4" customHeight="1">
+        <v>333</v>
+      </c>
+      <c r="F48" s="15"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
       <c r="B49" s="14" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>335</v>
+        <v>262</v>
       </c>
       <c r="F49" s="14" t="s">
         <v>336</v>
@@ -7120,41 +7141,41 @@
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="C50" s="15" t="s">
         <v>337</v>
       </c>
-      <c r="C50" s="15" t="s">
+      <c r="D50" s="15" t="s">
         <v>338</v>
       </c>
-      <c r="D50" s="15" t="s">
+      <c r="E50" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="F50" s="15" t="s">
         <v>339</v>
-      </c>
-      <c r="E50" s="15" t="s">
-        <v>240</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="51" ht="32.4" customHeight="1">
       <c r="B51" s="14" t="s">
-        <v>337</v>
+        <v>318</v>
       </c>
       <c r="C51" s="14" t="s">
+        <v>340</v>
+      </c>
+      <c r="D51" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="D51" s="14" t="s">
+      <c r="E51" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="E51" s="14" t="s">
+      <c r="F51" s="14" t="s">
         <v>343</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="15" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C52" s="15" t="s">
         <v>345</v>
@@ -7163,32 +7184,32 @@
         <v>346</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>206</v>
+        <v>240</v>
       </c>
       <c r="F52" s="15" t="s">
         <v>347</v>
       </c>
     </row>
-    <row r="53" ht="18" customHeight="1">
+    <row r="53" ht="32.4" customHeight="1">
       <c r="B53" s="14" t="s">
+        <v>344</v>
+      </c>
+      <c r="C53" s="14" t="s">
         <v>348</v>
       </c>
-      <c r="C53" s="14" t="s">
+      <c r="D53" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="D53" s="14" t="s">
+      <c r="E53" s="14" t="s">
         <v>350</v>
-      </c>
-      <c r="E53" s="14" t="s">
-        <v>240</v>
       </c>
       <c r="F53" s="14" t="s">
         <v>351</v>
       </c>
     </row>
-    <row r="54" ht="32.4" customHeight="1">
+    <row r="54" ht="18" customHeight="1">
       <c r="B54" s="15" t="s">
-        <v>348</v>
+        <v>344</v>
       </c>
       <c r="C54" s="15" t="s">
         <v>352</v>
@@ -7197,32 +7218,32 @@
         <v>353</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>240</v>
+        <v>206</v>
       </c>
       <c r="F54" s="15" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="55" ht="32.4" customHeight="1">
+    <row r="55" ht="18" customHeight="1">
       <c r="B55" s="14" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E55" s="14" t="s">
         <v>240</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="56" ht="32.4" customHeight="1">
       <c r="B56" s="15" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C56" s="15" t="s">
         <v>359</v>
@@ -7231,32 +7252,32 @@
         <v>360</v>
       </c>
       <c r="E56" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="F56" s="15" t="s">
         <v>361</v>
       </c>
-      <c r="F56" s="15" t="s">
+    </row>
+    <row r="57" ht="32.4" customHeight="1">
+      <c r="B57" s="14" t="s">
+        <v>355</v>
+      </c>
+      <c r="C57" s="14" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="B57" s="14" t="s">
-        <v>358</v>
-      </c>
-      <c r="C57" s="14" t="s">
+      <c r="D57" s="14" t="s">
         <v>363</v>
-      </c>
-      <c r="D57" s="14" t="s">
-        <v>364</v>
       </c>
       <c r="E57" s="14" t="s">
         <v>240</v>
       </c>
       <c r="F57" s="14" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="58" ht="32.4" customHeight="1">
+      <c r="B58" s="15" t="s">
         <v>365</v>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="B58" s="15" t="s">
-        <v>358</v>
       </c>
       <c r="C58" s="15" t="s">
         <v>366</v>
@@ -7265,92 +7286,92 @@
         <v>367</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>240</v>
+        <v>368</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="B59" s="14" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E59" s="14" t="s">
         <v>240</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="B60" s="15" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E60" s="15" t="s">
         <v>240</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="B61" s="14" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E61" s="14" t="s">
         <v>240</v>
       </c>
       <c r="F61" s="14" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="15" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E62" s="15" t="s">
         <v>240</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="14" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E63" s="14" t="s">
-        <v>383</v>
+        <v>240</v>
       </c>
       <c r="F63" s="14" t="s">
         <v>384</v>
@@ -7358,7 +7379,7 @@
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="B64" s="15" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C64" s="15" t="s">
         <v>385</v>
@@ -7367,30 +7388,64 @@
         <v>386</v>
       </c>
       <c r="E64" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="F64" s="15" t="s">
         <v>387</v>
-      </c>
-      <c r="F64" s="15" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="B65" s="14" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C65" s="14" t="s">
+        <v>388</v>
+      </c>
+      <c r="D65" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="D65" s="14" t="s">
+      <c r="E65" s="14" t="s">
         <v>390</v>
-      </c>
-      <c r="E65" s="14" t="s">
-        <v>231</v>
       </c>
       <c r="F65" s="14" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="66" ht="6" customHeight="1"/>
+    <row r="66" ht="18" customHeight="1">
+      <c r="B66" s="15" t="s">
+        <v>365</v>
+      </c>
+      <c r="C66" s="15" t="s">
+        <v>392</v>
+      </c>
+      <c r="D66" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="E66" s="15" t="s">
+        <v>394</v>
+      </c>
+      <c r="F66" s="15" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="B67" s="14" t="s">
+        <v>365</v>
+      </c>
+      <c r="C67" s="14" t="s">
+        <v>396</v>
+      </c>
+      <c r="D67" s="14" t="s">
+        <v>397</v>
+      </c>
+      <c r="E67" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="F67" s="14" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="68" ht="6" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B1:F1"/>
@@ -7432,7 +7487,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="6" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -7441,16 +7496,16 @@
     <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>161</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" ht="32.4" customHeight="1">
@@ -7459,7 +7514,7 @@
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="14" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>7</v>
@@ -7467,198 +7522,198 @@
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C7" s="15"/>
       <c r="D7" s="15" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="15" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
     </row>
     <row r="10" ht="32.4" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
     </row>
     <row r="11" ht="32.4" customHeight="1">
       <c r="B11" s="15" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="B13" s="15" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C13" s="15"/>
       <c r="D13" s="15" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="14" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
     </row>
     <row r="15" ht="32.4" customHeight="1">
       <c r="B15" s="15" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="C15" s="15"/>
       <c r="D15" s="15" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
     </row>
     <row r="16" ht="32.4" customHeight="1">
       <c r="B16" s="14" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="15" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C17" s="15"/>
       <c r="D17" s="15" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="14" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="14" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="15" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="C19" s="15"/>
       <c r="D19" s="15" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="14" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="C20" s="14"/>
       <c r="D20" s="14" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="15" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="C21" s="15"/>
       <c r="D21" s="15" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="E21" s="15" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
     </row>
     <row r="22" ht="32.4" customHeight="1">
       <c r="B22" s="14" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
@@ -7667,7 +7722,7 @@
       </c>
       <c r="C23" s="15"/>
       <c r="D23" s="15" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="E23" s="15"/>
     </row>
@@ -7675,7 +7730,7 @@
     <row r="25" ht="8" customHeight="1"/>
     <row r="26" ht="24" customHeight="1">
       <c r="B26" s="4" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -7684,7 +7739,7 @@
     <row r="27" ht="4" customHeight="1"/>
     <row r="28" ht="32.4" customHeight="1">
       <c r="B28" s="7" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
@@ -7692,7 +7747,7 @@
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
@@ -7700,7 +7755,7 @@
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="7" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
@@ -7708,7 +7763,7 @@
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="7" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="C31" s="7"/>
       <c r="D31" s="7"/>
@@ -7716,7 +7771,7 @@
     </row>
     <row r="32" ht="32.4" customHeight="1">
       <c r="B32" s="7" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
@@ -7724,7 +7779,7 @@
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="7" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="7"/>
@@ -7732,7 +7787,7 @@
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="B34" s="7" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="C34" s="7"/>
       <c r="D34" s="7"/>
@@ -7742,7 +7797,7 @@
     <row r="36" ht="8" customHeight="1"/>
     <row r="37" ht="24" customHeight="1">
       <c r="B37" s="4" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
@@ -7751,61 +7806,61 @@
     <row r="38" ht="4" customHeight="1"/>
     <row r="39" ht="18" customHeight="1">
       <c r="B39" s="13" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="E39" s="13"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="B40" s="14" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="E40" s="14"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="B41" s="15" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="E41" s="15"/>
     </row>
     <row r="42" ht="32.4" customHeight="1">
       <c r="B42" s="14" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="E42" s="14"/>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="15" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="E43" s="15"/>
     </row>
@@ -7863,7 +7918,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="6" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
@@ -7872,7 +7927,7 @@
     <row r="4" ht="6" customHeight="1"/>
     <row r="5" ht="16.2" customHeight="1">
       <c r="B5" s="9" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
@@ -7880,7 +7935,7 @@
     </row>
     <row r="6" ht="16.2" customHeight="1">
       <c r="B6" s="10" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
@@ -7888,7 +7943,7 @@
     </row>
     <row r="7" ht="16.2" customHeight="1">
       <c r="B7" s="10" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
@@ -7896,7 +7951,7 @@
     </row>
     <row r="8" ht="16.2" customHeight="1">
       <c r="B8" s="10" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -7904,7 +7959,7 @@
     </row>
     <row r="9" ht="16.2" customHeight="1">
       <c r="B9" s="10" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
@@ -7912,7 +7967,7 @@
     </row>
     <row r="10" ht="16.2" customHeight="1">
       <c r="B10" s="10" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
@@ -7920,7 +7975,7 @@
     </row>
     <row r="11" ht="16.2" customHeight="1">
       <c r="B11" s="10" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="10"/>
@@ -7928,7 +7983,7 @@
     </row>
     <row r="12" ht="16.2" customHeight="1">
       <c r="B12" s="10" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -7936,7 +7991,7 @@
     </row>
     <row r="13" ht="16.2" customHeight="1">
       <c r="B13" s="10" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -7944,7 +7999,7 @@
     </row>
     <row r="14" ht="16.2" customHeight="1">
       <c r="B14" s="10" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -7952,7 +8007,7 @@
     </row>
     <row r="15" ht="16.2" customHeight="1">
       <c r="B15" s="10" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -7960,7 +8015,7 @@
     </row>
     <row r="16" ht="16.2" customHeight="1">
       <c r="B16" s="10" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -7968,7 +8023,7 @@
     </row>
     <row r="17" ht="16.2" customHeight="1">
       <c r="B17" s="10" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
@@ -7976,7 +8031,7 @@
     </row>
     <row r="18" ht="16.2" customHeight="1">
       <c r="B18" s="10" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
@@ -7984,7 +8039,7 @@
     </row>
     <row r="19" ht="16.2" customHeight="1">
       <c r="B19" s="10" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
@@ -7992,7 +8047,7 @@
     </row>
     <row r="20" ht="16.2" customHeight="1">
       <c r="B20" s="10" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -8000,7 +8055,7 @@
     </row>
     <row r="21" ht="16.2" customHeight="1">
       <c r="B21" s="10" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
@@ -8008,7 +8063,7 @@
     </row>
     <row r="22" ht="16.2" customHeight="1">
       <c r="B22" s="10" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -8016,7 +8071,7 @@
     </row>
     <row r="23" ht="16.2" customHeight="1">
       <c r="B23" s="10" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
@@ -8024,7 +8079,7 @@
     </row>
     <row r="24" ht="16.2" customHeight="1">
       <c r="B24" s="10" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -8032,7 +8087,7 @@
     </row>
     <row r="25" ht="16.2" customHeight="1">
       <c r="B25" s="10" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -8040,7 +8095,7 @@
     </row>
     <row r="26" ht="16.2" customHeight="1">
       <c r="B26" s="10" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -8048,7 +8103,7 @@
     </row>
     <row r="27" ht="16.2" customHeight="1">
       <c r="B27" s="10" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -8056,7 +8111,7 @@
     </row>
     <row r="28" ht="16.2" customHeight="1">
       <c r="B28" s="10" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -8064,7 +8119,7 @@
     </row>
     <row r="29" ht="16.2" customHeight="1">
       <c r="B29" s="10" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
@@ -8072,7 +8127,7 @@
     </row>
     <row r="30" ht="16.2" customHeight="1">
       <c r="B30" s="10" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
@@ -8080,7 +8135,7 @@
     </row>
     <row r="31" ht="16.2" customHeight="1">
       <c r="B31" s="10" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
@@ -8088,7 +8143,7 @@
     </row>
     <row r="32" ht="16.2" customHeight="1">
       <c r="B32" s="10" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10"/>
@@ -8096,7 +8151,7 @@
     </row>
     <row r="33" ht="16.2" customHeight="1">
       <c r="B33" s="10" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
@@ -8104,7 +8159,7 @@
     </row>
     <row r="34" ht="16.2" customHeight="1">
       <c r="B34" s="10" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
@@ -8112,7 +8167,7 @@
     </row>
     <row r="35" ht="16.2" customHeight="1">
       <c r="B35" s="10" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
@@ -8120,7 +8175,7 @@
     </row>
     <row r="36" ht="16.2" customHeight="1">
       <c r="B36" s="10" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="C36" s="10"/>
       <c r="D36" s="10"/>
@@ -8128,7 +8183,7 @@
     </row>
     <row r="37" ht="16.2" customHeight="1">
       <c r="B37" s="10" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
@@ -8136,7 +8191,7 @@
     </row>
     <row r="38" ht="16.2" customHeight="1">
       <c r="B38" s="10" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
@@ -8144,7 +8199,7 @@
     </row>
     <row r="39" ht="16.2" customHeight="1">
       <c r="B39" s="10" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
@@ -8152,7 +8207,7 @@
     </row>
     <row r="40" ht="16.2" customHeight="1">
       <c r="B40" s="11" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
@@ -8162,7 +8217,7 @@
     <row r="42" ht="8" customHeight="1"/>
     <row r="43" ht="24" customHeight="1">
       <c r="B43" s="4" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -8171,401 +8226,401 @@
     <row r="44" ht="4" customHeight="1"/>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="13" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
     </row>
     <row r="46" ht="32.4" customHeight="1">
       <c r="B46" s="14" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
     </row>
     <row r="47" ht="32.4" customHeight="1">
       <c r="B47" s="15" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="14" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
     </row>
     <row r="49" ht="32.4" customHeight="1">
       <c r="B49" s="15" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="E49" s="15" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="B50" s="14" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="15" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="E51" s="15" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="14" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="53" ht="32.4" customHeight="1">
       <c r="B53" s="15" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="E53" s="15" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="14" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="15" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="14" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="B57" s="15" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="C57" s="15" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
       <c r="E57" s="15" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
     </row>
     <row r="58" ht="32.4" customHeight="1">
       <c r="B58" s="14" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="E58" s="14" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
     </row>
     <row r="59" ht="32.4" customHeight="1">
       <c r="B59" s="15" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
     </row>
     <row r="60" ht="32.4" customHeight="1">
       <c r="B60" s="14" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="D60" s="14" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="E60" s="14" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="B61" s="15" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
       <c r="C61" s="15" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="E61" s="15" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="B62" s="14" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
       <c r="E62" s="14" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="B63" s="15" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
     </row>
     <row r="64" ht="32.4" customHeight="1">
       <c r="B64" s="14" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
       <c r="D64" s="14" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
       <c r="E64" s="14" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
     </row>
     <row r="65" ht="32.4" customHeight="1">
       <c r="B65" s="15" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
       <c r="E65" s="15" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
     </row>
     <row r="66" ht="32.4" customHeight="1">
       <c r="B66" s="14" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
       <c r="D66" s="14" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
       <c r="E66" s="14" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="B67" s="15" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="C67" s="15" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="E67" s="15" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="68" ht="32.4" customHeight="1">
       <c r="B68" s="14" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>595</v>
+        <v>602</v>
       </c>
       <c r="D68" s="14" t="s">
-        <v>596</v>
+        <v>603</v>
       </c>
       <c r="E68" s="14" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
     </row>
     <row r="69" ht="32.4" customHeight="1">
       <c r="B69" s="15" t="s">
-        <v>598</v>
+        <v>605</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>599</v>
+        <v>606</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>600</v>
+        <v>607</v>
       </c>
       <c r="E69" s="15" t="s">
-        <v>601</v>
+        <v>608</v>
       </c>
     </row>
     <row r="70" ht="32.4" customHeight="1">
       <c r="B70" s="14" t="s">
-        <v>602</v>
+        <v>609</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="D70" s="14" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="E70" s="14" t="s">
-        <v>604</v>
+        <v>611</v>
       </c>
     </row>
     <row r="71" ht="32.4" customHeight="1">
       <c r="B71" s="15" t="s">
-        <v>605</v>
+        <v>612</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>606</v>
+        <v>613</v>
       </c>
       <c r="E71" s="15" t="s">
-        <v>607</v>
+        <v>614</v>
       </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="B72" s="14" t="s">
-        <v>608</v>
+        <v>615</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>609</v>
+        <v>616</v>
       </c>
       <c r="D72" s="14" t="s">
-        <v>610</v>
+        <v>617</v>
       </c>
       <c r="E72" s="14" t="s">
-        <v>611</v>
+        <v>618</v>
       </c>
     </row>
     <row r="73" ht="6" customHeight="1"/>
     <row r="74" ht="8" customHeight="1"/>
     <row r="75" ht="24" customHeight="1">
       <c r="B75" s="4" t="s">
-        <v>612</v>
+        <v>619</v>
       </c>
       <c r="C75" s="4"/>
       <c r="D75" s="4"/>
@@ -8574,133 +8629,133 @@
     <row r="76" ht="4" customHeight="1"/>
     <row r="77" ht="18" customHeight="1">
       <c r="B77" s="13" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>613</v>
+        <v>620</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>614</v>
+        <v>621</v>
       </c>
       <c r="E77" s="13"/>
     </row>
     <row r="78" ht="18" customHeight="1">
       <c r="B78" s="14" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="D78" s="14" t="s">
-        <v>616</v>
+        <v>623</v>
       </c>
       <c r="E78" s="14"/>
     </row>
     <row r="79" ht="18" customHeight="1">
       <c r="B79" s="15" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>617</v>
+        <v>624</v>
       </c>
       <c r="E79" s="15"/>
     </row>
     <row r="80" ht="18" customHeight="1">
       <c r="B80" s="14" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="D80" s="14" t="s">
-        <v>618</v>
+        <v>625</v>
       </c>
       <c r="E80" s="14"/>
     </row>
     <row r="81" ht="32.4" customHeight="1">
       <c r="B81" s="15" t="s">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>620</v>
+        <v>627</v>
       </c>
       <c r="E81" s="15"/>
     </row>
     <row r="82" ht="32.4" customHeight="1">
       <c r="B82" s="14" t="s">
-        <v>621</v>
+        <v>628</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
       <c r="D82" s="14" t="s">
-        <v>622</v>
+        <v>629</v>
       </c>
       <c r="E82" s="14"/>
     </row>
     <row r="83" ht="18" customHeight="1">
       <c r="B83" s="15" t="s">
-        <v>623</v>
+        <v>630</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>624</v>
+        <v>631</v>
       </c>
       <c r="E83" s="15"/>
     </row>
     <row r="84" ht="18" customHeight="1">
       <c r="B84" s="14" t="s">
-        <v>625</v>
+        <v>632</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>626</v>
+        <v>633</v>
       </c>
       <c r="D84" s="14" t="s">
-        <v>627</v>
+        <v>634</v>
       </c>
       <c r="E84" s="14"/>
     </row>
     <row r="85" ht="18" customHeight="1">
       <c r="B85" s="15" t="s">
-        <v>628</v>
+        <v>635</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>629</v>
+        <v>636</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>630</v>
+        <v>637</v>
       </c>
       <c r="E85" s="15"/>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="B86" s="14" t="s">
-        <v>631</v>
+        <v>638</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>632</v>
+        <v>639</v>
       </c>
       <c r="D86" s="14" t="s">
-        <v>633</v>
+        <v>640</v>
       </c>
       <c r="E86" s="14"/>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="B87" s="15" t="s">
-        <v>634</v>
+        <v>641</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>635</v>
+        <v>642</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>636</v>
+        <v>643</v>
       </c>
       <c r="E87" s="15"/>
     </row>
@@ -8708,7 +8763,7 @@
     <row r="89" ht="8" customHeight="1"/>
     <row r="90" ht="24" customHeight="1">
       <c r="B90" s="4" t="s">
-        <v>637</v>
+        <v>644</v>
       </c>
       <c r="C90" s="4"/>
       <c r="D90" s="4"/>
@@ -8717,7 +8772,7 @@
     <row r="91" ht="4" customHeight="1"/>
     <row r="92" ht="18" customHeight="1">
       <c r="B92" s="7" t="s">
-        <v>638</v>
+        <v>645</v>
       </c>
       <c r="C92" s="7"/>
       <c r="D92" s="7"/>
@@ -8725,7 +8780,7 @@
     </row>
     <row r="93" ht="18" customHeight="1">
       <c r="B93" s="7" t="s">
-        <v>639</v>
+        <v>646</v>
       </c>
       <c r="C93" s="7"/>
       <c r="D93" s="7"/>
@@ -8733,7 +8788,7 @@
     </row>
     <row r="94" ht="18" customHeight="1">
       <c r="B94" s="7" t="s">
-        <v>640</v>
+        <v>647</v>
       </c>
       <c r="C94" s="7"/>
       <c r="D94" s="7"/>
@@ -8741,7 +8796,7 @@
     </row>
     <row r="95" ht="18" customHeight="1">
       <c r="B95" s="7" t="s">
-        <v>641</v>
+        <v>648</v>
       </c>
       <c r="C95" s="7"/>
       <c r="D95" s="7"/>
@@ -8839,7 +8894,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>642</v>
+        <v>649</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -8847,42 +8902,42 @@
     <row r="4" ht="4" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="13" t="s">
-        <v>643</v>
+        <v>650</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>644</v>
+        <v>651</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>645</v>
+        <v>652</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="B6" s="14" t="s">
-        <v>646</v>
+        <v>653</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>647</v>
+        <v>654</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>648</v>
+        <v>655</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>649</v>
+        <v>656</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>650</v>
+        <v>657</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>651</v>
+        <v>658</v>
       </c>
     </row>
     <row r="8" ht="6" customHeight="1"/>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="24" customHeight="1">
       <c r="B10" s="4" t="s">
-        <v>652</v>
+        <v>659</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -8890,7 +8945,7 @@
     <row r="11" ht="4" customHeight="1"/>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="6" t="s">
-        <v>653</v>
+        <v>660</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -8905,42 +8960,42 @@
     </row>
     <row r="15" ht="16.2" customHeight="1">
       <c r="B15" s="10" t="s">
-        <v>654</v>
+        <v>661</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
     </row>
     <row r="16" ht="16.2" customHeight="1">
       <c r="B16" s="10" t="s">
-        <v>655</v>
+        <v>662</v>
       </c>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
     </row>
     <row r="17" ht="16.2" customHeight="1">
       <c r="B17" s="10" t="s">
-        <v>656</v>
+        <v>663</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
     </row>
     <row r="18" ht="16.2" customHeight="1">
       <c r="B18" s="10" t="s">
-        <v>657</v>
+        <v>664</v>
       </c>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
     </row>
     <row r="19" ht="16.2" customHeight="1">
       <c r="B19" s="10" t="s">
-        <v>658</v>
+        <v>665</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
     </row>
     <row r="20" ht="16.2" customHeight="1">
       <c r="B20" s="11" t="s">
-        <v>659</v>
+        <v>666</v>
       </c>
       <c r="C20" s="11"/>
       <c r="D20" s="11"/>
@@ -8955,21 +9010,21 @@
     </row>
     <row r="23" ht="16.2" customHeight="1">
       <c r="B23" s="10" t="s">
-        <v>660</v>
+        <v>667</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
     </row>
     <row r="24" ht="16.2" customHeight="1">
       <c r="B24" s="10" t="s">
-        <v>661</v>
+        <v>668</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
     </row>
     <row r="25" ht="16.2" customHeight="1">
       <c r="B25" s="11" t="s">
-        <v>662</v>
+        <v>669</v>
       </c>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
@@ -8988,68 +9043,68 @@
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="14" t="s">
-        <v>663</v>
+        <v>670</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>664</v>
+        <v>671</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>665</v>
+        <v>672</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="15" t="s">
-        <v>666</v>
+        <v>673</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>667</v>
+        <v>674</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>668</v>
+        <v>675</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="14" t="s">
-        <v>669</v>
+        <v>676</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>670</v>
+        <v>677</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>671</v>
+        <v>678</v>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="15" t="s">
-        <v>672</v>
+        <v>679</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>673</v>
+        <v>680</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>674</v>
+        <v>681</v>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="B32" s="14" t="s">
-        <v>675</v>
+        <v>682</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>676</v>
+        <v>683</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>677</v>
+        <v>684</v>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="B33" s="15" t="s">
-        <v>678</v>
+        <v>685</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>680</v>
+        <v>687</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
@@ -9060,58 +9115,58 @@
         <v>169</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>681</v>
+        <v>688</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="15" t="s">
-        <v>682</v>
+        <v>689</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>683</v>
+        <v>690</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>684</v>
+        <v>691</v>
       </c>
     </row>
     <row r="36" ht="32.4" customHeight="1">
       <c r="B36" s="14" t="s">
-        <v>685</v>
+        <v>692</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>686</v>
+        <v>693</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>687</v>
+        <v>694</v>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="B37" s="15" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>689</v>
+        <v>696</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>690</v>
+        <v>697</v>
       </c>
     </row>
     <row r="38" ht="32.4" customHeight="1">
       <c r="B38" s="14" t="s">
-        <v>691</v>
+        <v>698</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>692</v>
+        <v>699</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>693</v>
+        <v>700</v>
       </c>
     </row>
     <row r="39" ht="6" customHeight="1"/>
     <row r="40" ht="8" customHeight="1"/>
     <row r="41" ht="24" customHeight="1">
       <c r="B41" s="4" t="s">
-        <v>694</v>
+        <v>701</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
@@ -9119,7 +9174,7 @@
     <row r="42" ht="4" customHeight="1"/>
     <row r="43" ht="18" customHeight="1">
       <c r="B43" s="13" t="s">
-        <v>695</v>
+        <v>702</v>
       </c>
       <c r="C43" s="13" t="s">
         <v>194</v>
@@ -9130,152 +9185,152 @@
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="B44" s="14" t="s">
-        <v>696</v>
+        <v>703</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>698</v>
+        <v>705</v>
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="15" t="s">
-        <v>699</v>
+        <v>706</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>700</v>
+        <v>707</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="14" t="s">
-        <v>702</v>
+        <v>709</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>703</v>
+        <v>710</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>704</v>
+        <v>711</v>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="15" t="s">
-        <v>705</v>
+        <v>712</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>707</v>
+        <v>714</v>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="B48" s="14" t="s">
-        <v>708</v>
+        <v>715</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>709</v>
+        <v>716</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>710</v>
+        <v>717</v>
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="B49" s="15" t="s">
-        <v>615</v>
+        <v>622</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>711</v>
+        <v>718</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>712</v>
+        <v>719</v>
       </c>
     </row>
     <row r="50" ht="32.4" customHeight="1">
       <c r="B50" s="14" t="s">
-        <v>713</v>
+        <v>720</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>714</v>
+        <v>721</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>715</v>
+        <v>722</v>
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="B51" s="15" t="s">
-        <v>716</v>
+        <v>723</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>717</v>
+        <v>724</v>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="B52" s="14" t="s">
-        <v>718</v>
+        <v>725</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>720</v>
+        <v>727</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="B53" s="15" t="s">
-        <v>721</v>
+        <v>728</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>722</v>
+        <v>729</v>
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="B54" s="14" t="s">
-        <v>723</v>
+        <v>730</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>724</v>
+        <v>731</v>
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="B55" s="15" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="B56" s="14" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>729</v>
+        <v>736</v>
       </c>
     </row>
     <row r="57" ht="6" customHeight="1"/>
     <row r="58" ht="8" customHeight="1"/>
     <row r="59" ht="24" customHeight="1">
       <c r="B59" s="4" t="s">
-        <v>730</v>
+        <v>737</v>
       </c>
       <c r="C59" s="4"/>
       <c r="D59" s="4"/>
@@ -9283,21 +9338,21 @@
     <row r="60" ht="4" customHeight="1"/>
     <row r="61" ht="16.2" customHeight="1">
       <c r="B61" s="9" t="s">
-        <v>731</v>
+        <v>738</v>
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="9"/>
     </row>
     <row r="62" ht="16.2" customHeight="1">
       <c r="B62" s="10" t="s">
-        <v>732</v>
+        <v>739</v>
       </c>
       <c r="C62" s="10"/>
       <c r="D62" s="10"/>
     </row>
     <row r="63" ht="16.2" customHeight="1">
       <c r="B63" s="11" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="C63" s="11"/>
       <c r="D63" s="11"/>
@@ -9312,7 +9367,7 @@
     </row>
     <row r="66" ht="30.6" customHeight="1">
       <c r="B66" s="11" t="s">
-        <v>734</v>
+        <v>741</v>
       </c>
       <c r="C66" s="11"/>
       <c r="D66" s="11"/>
@@ -9320,14 +9375,14 @@
     <row r="67" ht="6" customHeight="1"/>
     <row r="68" ht="18" customHeight="1">
       <c r="B68" s="7" t="s">
-        <v>735</v>
+        <v>742</v>
       </c>
       <c r="C68" s="7"/>
       <c r="D68" s="7"/>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="B69" s="7" t="s">
-        <v>736</v>
+        <v>743</v>
       </c>
       <c r="C69" s="7"/>
       <c r="D69" s="7"/>
@@ -9336,7 +9391,7 @@
     <row r="71" ht="8" customHeight="1"/>
     <row r="72" ht="24" customHeight="1">
       <c r="B72" s="4" t="s">
-        <v>737</v>
+        <v>744</v>
       </c>
       <c r="C72" s="4"/>
       <c r="D72" s="4"/>
@@ -9344,21 +9399,21 @@
     <row r="73" ht="4" customHeight="1"/>
     <row r="74" ht="18" customHeight="1">
       <c r="B74" s="7" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="C74" s="7"/>
       <c r="D74" s="7"/>
     </row>
     <row r="75" ht="18" customHeight="1">
       <c r="B75" s="7" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
     </row>
     <row r="76" ht="18" customHeight="1">
       <c r="B76" s="7" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="C76" s="7"/>
       <c r="D76" s="7"/>
@@ -9427,7 +9482,7 @@
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="4" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -9435,7 +9490,7 @@
     <row r="4" ht="4" customHeight="1"/>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="6" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
@@ -9443,75 +9498,75 @@
     <row r="6" ht="6" customHeight="1"/>
     <row r="7" ht="18" customHeight="1">
       <c r="B7" s="13" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="14" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="B9" s="15" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="B10" s="14" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="15" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="B12" s="14" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
     </row>
     <row r="13" ht="6" customHeight="1"/>
     <row r="14" ht="8" customHeight="1"/>
     <row r="15" ht="24" customHeight="1">
       <c r="B15" s="4" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
@@ -9519,49 +9574,49 @@
     <row r="16" ht="4" customHeight="1"/>
     <row r="17" ht="18" customHeight="1">
       <c r="B17" s="7" t="s">
-        <v>762</v>
+        <v>769</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="B18" s="7" t="s">
-        <v>763</v>
+        <v>770</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="7" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="B20" s="7" t="s">
-        <v>765</v>
+        <v>772</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="B21" s="7" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="B22" s="7" t="s">
-        <v>767</v>
+        <v>774</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="B23" s="7" t="s">
-        <v>768</v>
+        <v>775</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="7"/>
@@ -9570,7 +9625,7 @@
     <row r="25" ht="8" customHeight="1"/>
     <row r="26" ht="24" customHeight="1">
       <c r="B26" s="4" t="s">
-        <v>769</v>
+        <v>776</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
@@ -9578,53 +9633,53 @@
     <row r="27" ht="4" customHeight="1"/>
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="13" t="s">
-        <v>770</v>
+        <v>777</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>771</v>
+        <v>778</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>772</v>
+        <v>779</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="14" t="s">
-        <v>773</v>
+        <v>780</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>775</v>
+        <v>782</v>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="B30" s="15" t="s">
-        <v>776</v>
+        <v>783</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>777</v>
+        <v>784</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>778</v>
+        <v>785</v>
       </c>
     </row>
     <row r="31" ht="32.4" customHeight="1">
       <c r="B31" s="14" t="s">
-        <v>779</v>
+        <v>786</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>780</v>
+        <v>787</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>781</v>
+        <v>788</v>
       </c>
     </row>
     <row r="32" ht="6" customHeight="1"/>
     <row r="33" ht="8" customHeight="1"/>
     <row r="34" ht="24" customHeight="1">
       <c r="B34" s="4" t="s">
-        <v>782</v>
+        <v>789</v>
       </c>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
@@ -9632,35 +9687,35 @@
     <row r="35" ht="4" customHeight="1"/>
     <row r="36" ht="16.2" customHeight="1">
       <c r="B36" s="9" t="s">
-        <v>783</v>
+        <v>790</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
     </row>
     <row r="37" ht="16.2" customHeight="1">
       <c r="B37" s="10" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="10"/>
     </row>
     <row r="38" ht="16.2" customHeight="1">
       <c r="B38" s="10" t="s">
-        <v>785</v>
+        <v>792</v>
       </c>
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
     </row>
     <row r="39" ht="16.2" customHeight="1">
       <c r="B39" s="10" t="s">
-        <v>786</v>
+        <v>793</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" ht="16.2" customHeight="1">
       <c r="B40" s="11" t="s">
-        <v>787</v>
+        <v>794</v>
       </c>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
@@ -9669,7 +9724,7 @@
     <row r="42" ht="8" customHeight="1"/>
     <row r="43" ht="24" customHeight="1">
       <c r="B43" s="4" t="s">
-        <v>788</v>
+        <v>795</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
@@ -9677,21 +9732,21 @@
     <row r="44" ht="4" customHeight="1"/>
     <row r="45" ht="18" customHeight="1">
       <c r="B45" s="7" t="s">
-        <v>789</v>
+        <v>796</v>
       </c>
       <c r="C45" s="7"/>
       <c r="D45" s="7"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="B46" s="7" t="s">
-        <v>790</v>
+        <v>797</v>
       </c>
       <c r="C46" s="7"/>
       <c r="D46" s="7"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="B47" s="7" t="s">
-        <v>791</v>
+        <v>798</v>
       </c>
       <c r="C47" s="7"/>
       <c r="D47" s="7"/>
@@ -9700,7 +9755,7 @@
     <row r="49" ht="8" customHeight="1"/>
     <row r="50" ht="24" customHeight="1">
       <c r="B50" s="4" t="s">
-        <v>792</v>
+        <v>799</v>
       </c>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
@@ -9708,7 +9763,7 @@
     <row r="51" ht="4" customHeight="1"/>
     <row r="52" ht="46.8" customHeight="1">
       <c r="B52" s="6" t="s">
-        <v>793</v>
+        <v>800</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="6"/>

</xml_diff>